<commit_message>
add long and lat
</commit_message>
<xml_diff>
--- a/data/intern/pumping_stations_belgium.xlsx
+++ b/data/intern/pumping_stations_belgium.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12450"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="7890" windowHeight="1320"/>
   </bookViews>
   <sheets>
     <sheet name="pumping_stations_belgium" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="191">
   <si>
     <t>Name</t>
   </si>
@@ -40,6 +40,12 @@
   </si>
   <si>
     <t>Discharge.into.freshwater.or.estuary.sea</t>
+  </si>
+  <si>
+    <t>Longitude</t>
+  </si>
+  <si>
+    <t>Latitude</t>
   </si>
   <si>
     <t>Baasrode</t>
@@ -1392,10 +1398,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G173"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:I173"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1417,10 +1423,16 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B2">
         <v>135370</v>
@@ -1435,15 +1447,21 @@
         <v>3</v>
       </c>
       <c r="F2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H2">
+        <v>4.1601375873968101</v>
+      </c>
+      <c r="I2">
+        <v>51.045218729644603</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3">
         <v>26825</v>
@@ -1458,15 +1476,21 @@
         <v>1</v>
       </c>
       <c r="F3" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G3" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H3">
+        <v>2.61199269657219</v>
+      </c>
+      <c r="I3">
+        <v>51.049959187899702</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4">
         <v>146987</v>
@@ -1481,15 +1505,21 @@
         <v>4</v>
       </c>
       <c r="F4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G4" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H4">
+        <v>4.3257141247055699</v>
+      </c>
+      <c r="I4">
+        <v>51.130321111090701</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5">
         <v>104189</v>
@@ -1504,15 +1534,21 @@
         <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H5">
+        <v>3.7123305951790102</v>
+      </c>
+      <c r="I5">
+        <v>51.271599628743999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>44344</v>
@@ -1527,15 +1563,21 @@
         <v>1</v>
       </c>
       <c r="F6" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H6">
+        <v>2.8669143210463002</v>
+      </c>
+      <c r="I6">
+        <v>50.893381039066</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>43177</v>
@@ -1550,15 +1592,21 @@
         <v>1</v>
       </c>
       <c r="F7" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H7">
+        <v>2.8497718371724701</v>
+      </c>
+      <c r="I7">
+        <v>50.910450742195898</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>116569</v>
@@ -1573,15 +1621,21 @@
         <v>1</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H8">
+        <v>3.8910168745657101</v>
+      </c>
+      <c r="I8">
+        <v>51.145670251277501</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>116607</v>
@@ -1596,15 +1650,21 @@
         <v>2</v>
       </c>
       <c r="F9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G9" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H9">
+        <v>3.8915575075934599</v>
+      </c>
+      <c r="I9">
+        <v>51.145906144400797</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>82539</v>
@@ -1619,15 +1679,21 @@
         <v>4</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G10" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H10">
+        <v>3.4128351431056698</v>
+      </c>
+      <c r="I10">
+        <v>50.747749425107003</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>54304</v>
@@ -1642,15 +1708,21 @@
         <v>1</v>
       </c>
       <c r="F11" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G11" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H11">
+        <v>3.0009434657947902</v>
+      </c>
+      <c r="I11">
+        <v>51.1531369740404</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>29108</v>
@@ -1665,15 +1737,21 @@
         <v>2</v>
       </c>
       <c r="F12" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G12" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H12">
+        <v>2.6448042375616598</v>
+      </c>
+      <c r="I12">
+        <v>51.043313665965599</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>149076</v>
@@ -1688,15 +1766,21 @@
         <v>3</v>
       </c>
       <c r="F13" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H13">
+        <v>4.3555359262754196</v>
+      </c>
+      <c r="I13">
+        <v>51.207440945303901</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>50088</v>
@@ -1711,15 +1795,21 @@
         <v>2</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="H14">
+        <v>2.9386810371198302</v>
+      </c>
+      <c r="I14">
+        <v>51.2182885077099</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B15">
         <v>43083</v>
@@ -1734,15 +1824,21 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H15">
+        <v>2.8411047260743798</v>
+      </c>
+      <c r="I15">
+        <v>51.135767850770797</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B16">
         <v>122774</v>
@@ -1757,15 +1853,21 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H16">
+        <v>3.97988614496898</v>
+      </c>
+      <c r="I16">
+        <v>51.121977849593399</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B17">
         <v>75234</v>
@@ -1780,15 +1882,21 @@
         <v>1</v>
       </c>
       <c r="F17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G17" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H17">
+        <v>3.29751863265377</v>
+      </c>
+      <c r="I17">
+        <v>51.266866728979103</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B18">
         <v>109670</v>
@@ -1803,15 +1911,21 @@
         <v>4</v>
       </c>
       <c r="F18" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G18" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H18">
+        <v>3.7937524567669998</v>
+      </c>
+      <c r="I18">
+        <v>51.037808529582698</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B19">
         <v>114791</v>
@@ -1826,15 +1940,21 @@
         <v>2</v>
       </c>
       <c r="F19" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G19" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H19">
+        <v>3.8697013258417101</v>
+      </c>
+      <c r="I19">
+        <v>50.7620667673038</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B20">
         <v>64351</v>
@@ -1849,15 +1969,21 @@
         <v>2</v>
       </c>
       <c r="F20" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G20" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H20">
+        <v>3.1430327881384699</v>
+      </c>
+      <c r="I20">
+        <v>51.211431167209398</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B21">
         <v>61006</v>
@@ -1872,15 +1998,21 @@
         <v>3</v>
       </c>
       <c r="F21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G21" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H21">
+        <v>3.0953707698195698</v>
+      </c>
+      <c r="I21">
+        <v>51.203627921198297</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B22">
         <v>114489</v>
@@ -1895,15 +2027,21 @@
         <v>1</v>
       </c>
       <c r="F22" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G22" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H22">
+        <v>3.8612706849204401</v>
+      </c>
+      <c r="I22">
+        <v>51.1476856385788</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B23">
         <v>187646</v>
@@ -1918,15 +2056,21 @@
         <v>3</v>
       </c>
       <c r="F23" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G23" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H23">
+        <v>4.9073371097229801</v>
+      </c>
+      <c r="I23">
+        <v>51.198148570443699</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B24">
         <v>129267</v>
@@ -1941,15 +2085,21 @@
         <v>4</v>
       </c>
       <c r="F24" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G24" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H24">
+        <v>4.0733050387435199</v>
+      </c>
+      <c r="I24">
+        <v>51.014407646080102</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B25">
         <v>110541</v>
@@ -1964,15 +2114,21 @@
         <v>2</v>
       </c>
       <c r="F25" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G25" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H25">
+        <v>3.8057451265094202</v>
+      </c>
+      <c r="I25">
+        <v>51.073256841163399</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B26">
         <v>129000</v>
@@ -1987,15 +2143,21 @@
         <v>2</v>
       </c>
       <c r="F26" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G26" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H26">
+        <v>4.0689111126376201</v>
+      </c>
+      <c r="I26">
+        <v>51.106641557632301</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B27">
         <v>54230</v>
@@ -2010,15 +2172,21 @@
         <v>2</v>
       </c>
       <c r="F27" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G27" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H27">
+        <v>2.9999260262341498</v>
+      </c>
+      <c r="I27">
+        <v>51.151758684495199</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B28">
         <v>54231</v>
@@ -2033,15 +2201,21 @@
         <v>1</v>
       </c>
       <c r="F28" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G28" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H28">
+        <v>2.9999403158975699</v>
+      </c>
+      <c r="I28">
+        <v>51.151758850106198</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B29">
         <v>156614</v>
@@ -2056,15 +2230,21 @@
         <v>4</v>
       </c>
       <c r="F29" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G29" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H29">
+        <v>4.4631273540082903</v>
+      </c>
+      <c r="I29">
+        <v>51.074496986649599</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B30">
         <v>92644</v>
@@ -2079,15 +2259,21 @@
         <v>3</v>
       </c>
       <c r="F30" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G30" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H30">
+        <v>3.5485804457625898</v>
+      </c>
+      <c r="I30">
+        <v>51.175844925975497</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B31">
         <v>170609</v>
@@ -2102,15 +2288,21 @@
         <v>2</v>
       </c>
       <c r="F31" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G31" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H31">
+        <v>4.6614187041470503</v>
+      </c>
+      <c r="I31">
+        <v>50.851766772863698</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B32">
         <v>107664</v>
@@ -2125,15 +2317,21 @@
         <v>7</v>
       </c>
       <c r="F32" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G32" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H32">
+        <v>3.7634973397610798</v>
+      </c>
+      <c r="I32">
+        <v>51.165886369095801</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B33">
         <v>47523</v>
@@ -2148,15 +2346,21 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G33" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H33">
+        <v>2.9076782819381499</v>
+      </c>
+      <c r="I33">
+        <v>51.035799196861603</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B34">
         <v>118357</v>
@@ -2171,15 +2375,21 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G34" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H34">
+        <v>3.9165378665499402</v>
+      </c>
+      <c r="I34">
+        <v>51.1488178330195</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B35">
         <v>124863</v>
@@ -2194,15 +2404,21 @@
         <v>6</v>
       </c>
       <c r="F35" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G35" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H35">
+        <v>4.00990902357991</v>
+      </c>
+      <c r="I35">
+        <v>51.097793881858102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B36">
         <v>137033</v>
@@ -2217,15 +2433,21 @@
         <v>3</v>
       </c>
       <c r="F36" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G36" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H36">
+        <v>4.1837641251589996</v>
+      </c>
+      <c r="I36">
+        <v>51.067361910739201</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B37">
         <v>169490</v>
@@ -2240,15 +2462,21 @@
         <v>2</v>
       </c>
       <c r="F37" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G37" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H37">
+        <v>4.6471541885680301</v>
+      </c>
+      <c r="I37">
+        <v>51.125657092329</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B38">
         <v>128245</v>
@@ -2263,15 +2491,21 @@
         <v>2</v>
       </c>
       <c r="F38" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G38" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H38">
+        <v>4.0589945233670797</v>
+      </c>
+      <c r="I38">
+        <v>50.976023059435697</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B39">
         <v>157852</v>
@@ -2286,15 +2520,21 @@
         <v>2</v>
       </c>
       <c r="F39" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G39" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H39">
+        <v>4.4807963489785596</v>
+      </c>
+      <c r="I39">
+        <v>51.076405030924903</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B40">
         <v>244197</v>
@@ -2309,15 +2549,21 @@
         <v>8</v>
       </c>
       <c r="F40" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G40" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H40">
+        <v>5.7105296178363698</v>
+      </c>
+      <c r="I40">
+        <v>50.992708452483697</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B41">
         <v>129846</v>
@@ -2332,15 +2578,21 @@
         <v>2</v>
       </c>
       <c r="F41" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G41" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H41">
+        <v>4.0810106610482704</v>
+      </c>
+      <c r="I41">
+        <v>51.103381708879802</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B42">
         <v>132542</v>
@@ -2355,15 +2607,21 @@
         <v>3</v>
       </c>
       <c r="F42" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G42" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H42">
+        <v>4.1198336669736104</v>
+      </c>
+      <c r="I42">
+        <v>51.041014728309797</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B43">
         <v>212378</v>
@@ -2378,15 +2636,21 @@
         <v>2</v>
       </c>
       <c r="F43" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G43" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H43">
+        <v>5.2583070840482904</v>
+      </c>
+      <c r="I43">
+        <v>51.047746205813702</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B44">
         <v>142905</v>
@@ -2401,15 +2665,21 @@
         <v>1</v>
       </c>
       <c r="F44" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G44" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H44">
+        <v>4.2681750498286801</v>
+      </c>
+      <c r="I44">
+        <v>50.768047224666098</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="B45">
         <v>126188</v>
@@ -2424,15 +2694,21 @@
         <v>2</v>
       </c>
       <c r="F45" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G45" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H45">
+        <v>4.0281889790476599</v>
+      </c>
+      <c r="I45">
+        <v>51.185200665172097</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B46">
         <v>146575</v>
@@ -2447,15 +2723,21 @@
         <v>1</v>
       </c>
       <c r="F46" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G46" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H46">
+        <v>4.3198643722627503</v>
+      </c>
+      <c r="I46">
+        <v>51.09553239513</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B47">
         <v>25214</v>
@@ -2470,15 +2752,21 @@
         <v>1</v>
       </c>
       <c r="F47" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G47" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H47">
+        <v>2.5900447453656898</v>
+      </c>
+      <c r="I47">
+        <v>51.02277208105</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B48">
         <v>24671</v>
@@ -2493,15 +2781,21 @@
         <v>2</v>
       </c>
       <c r="F48" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G48" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H48">
+        <v>2.5829457171364498</v>
+      </c>
+      <c r="I48">
+        <v>51.005922171723398</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B49">
         <v>154154</v>
@@ -2516,15 +2810,21 @@
         <v>4</v>
       </c>
       <c r="F49" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G49" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+      <c r="H49">
+        <v>4.4282384470636398</v>
+      </c>
+      <c r="I49">
+        <v>51.238948541341301</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B50">
         <v>161071</v>
@@ -2539,15 +2839,21 @@
         <v>2</v>
       </c>
       <c r="F50" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G50" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H50">
+        <v>4.5268355794780204</v>
+      </c>
+      <c r="I50">
+        <v>51.107938779109297</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B51">
         <v>48131</v>
@@ -2562,15 +2868,21 @@
         <v>2</v>
       </c>
       <c r="F51" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G51" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H51">
+        <v>2.9120553825809399</v>
+      </c>
+      <c r="I51">
+        <v>51.173803699508497</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B52">
         <v>48130</v>
@@ -2585,15 +2897,21 @@
         <v>1</v>
       </c>
       <c r="F52" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G52" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H52">
+        <v>2.91203996500326</v>
+      </c>
+      <c r="I52">
+        <v>51.173839470551101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B53">
         <v>116220</v>
@@ -2608,15 +2926,21 @@
         <v>2</v>
       </c>
       <c r="F53" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G53" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H53">
+        <v>3.88581743458262</v>
+      </c>
+      <c r="I53">
+        <v>51.166206508737801</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B54">
         <v>116954</v>
@@ -2631,15 +2955,21 @@
         <v>2</v>
       </c>
       <c r="F54" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G54" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H54">
+        <v>3.8962911510323202</v>
+      </c>
+      <c r="I54">
+        <v>51.168199372483798</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B55">
         <v>250360</v>
@@ -2654,15 +2984,21 @@
         <v>1</v>
       </c>
       <c r="F55" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G55" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H55">
+        <v>5.8034497710128399</v>
+      </c>
+      <c r="I55">
+        <v>51.1598873827378</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B56">
         <v>142903</v>
@@ -2677,15 +3013,21 @@
         <v>3</v>
       </c>
       <c r="F56" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G56" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H56">
+        <v>4.2671268313981496</v>
+      </c>
+      <c r="I56">
+        <v>51.2438014476527</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B57">
         <v>69887</v>
@@ -2700,15 +3042,21 @@
         <v>3</v>
       </c>
       <c r="F57" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G57" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H57">
+        <v>3.2226085315642798</v>
+      </c>
+      <c r="I57">
+        <v>51.197450303089603</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B58">
         <v>196336</v>
@@ -2723,15 +3071,21 @@
         <v>2</v>
       </c>
       <c r="F58" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G58" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H58">
+        <v>5.0338914816765303</v>
+      </c>
+      <c r="I58">
+        <v>51.354281526024003</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B59">
         <v>129249</v>
@@ -2746,15 +3100,21 @@
         <v>1</v>
       </c>
       <c r="F59" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G59" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H59">
+        <v>4.0724782019986296</v>
+      </c>
+      <c r="I59">
+        <v>51.104780871225103</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="B60">
         <v>215148</v>
@@ -2769,15 +3129,21 @@
         <v>2</v>
       </c>
       <c r="F60" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G60" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H60">
+        <v>5.29772813671251</v>
+      </c>
+      <c r="I60">
+        <v>51.043567118560802</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="B61">
         <v>130966</v>
@@ -2792,15 +3158,21 @@
         <v>1</v>
       </c>
       <c r="F61" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G61" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H61">
+        <v>4.0969876802441103</v>
+      </c>
+      <c r="I61">
+        <v>51.105738633644201</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B62">
         <v>125644</v>
@@ -2815,15 +3187,21 @@
         <v>3</v>
       </c>
       <c r="F62" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G62" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H62">
+        <v>4.0217055258125196</v>
+      </c>
+      <c r="I62">
+        <v>51.010437743458702</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B63">
         <v>37269</v>
@@ -2838,15 +3216,21 @@
         <v>2</v>
       </c>
       <c r="F63" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G63" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="H63">
+        <v>2.7580305904839499</v>
+      </c>
+      <c r="I63">
+        <v>51.135472788522897</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B64">
         <v>47411</v>
@@ -2861,15 +3245,21 @@
         <v>1</v>
       </c>
       <c r="F64" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G64" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H64">
+        <v>2.9014905545046101</v>
+      </c>
+      <c r="I64">
+        <v>51.182321639636299</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B65">
         <v>203259</v>
@@ -2884,15 +3274,21 @@
         <v>1</v>
       </c>
       <c r="F65" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G65" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H65">
+        <v>5.1306396529429898</v>
+      </c>
+      <c r="I65">
+        <v>51.193844371404197</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B66">
         <v>59734</v>
@@ -2907,15 +3303,21 @@
         <v>3</v>
       </c>
       <c r="F66" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G66" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H66">
+        <v>3.0772046096615502</v>
+      </c>
+      <c r="I66">
+        <v>51.202316161290597</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B67">
         <v>171030</v>
@@ -2930,15 +3332,21 @@
         <v>2</v>
       </c>
       <c r="F67" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G67" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H67">
+        <v>4.6694519791781701</v>
+      </c>
+      <c r="I67">
+        <v>51.172181719900202</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B68">
         <v>216370</v>
@@ -2953,15 +3361,21 @@
         <v>2</v>
       </c>
       <c r="F68" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G68" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H68">
+        <v>5.3143012513475698</v>
+      </c>
+      <c r="I68">
+        <v>51.001381035849597</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B69">
         <v>162224</v>
@@ -2976,15 +3390,21 @@
         <v>2</v>
       </c>
       <c r="F69" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G69" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H69">
+        <v>4.5433248474434897</v>
+      </c>
+      <c r="I69">
+        <v>51.114845779337699</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B70">
         <v>49012</v>
@@ -2999,15 +3419,21 @@
         <v>1</v>
       </c>
       <c r="F70" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G70" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H70">
+        <v>2.92553971107102</v>
+      </c>
+      <c r="I70">
+        <v>51.145182243097302</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B71">
         <v>112398</v>
@@ -3022,15 +3448,21 @@
         <v>3</v>
       </c>
       <c r="F71" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G71" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H71">
+        <v>3.8314018122425799</v>
+      </c>
+      <c r="I71">
+        <v>51.146465977781403</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B72">
         <v>113984</v>
@@ -3045,15 +3477,21 @@
         <v>3</v>
       </c>
       <c r="F72" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G72" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H72">
+        <v>3.8538689222309199</v>
+      </c>
+      <c r="I72">
+        <v>51.164462733058102</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B73">
         <v>105770</v>
@@ -3068,15 +3506,21 @@
         <v>1</v>
       </c>
       <c r="F73" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G73" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H73">
+        <v>3.7384877681391302</v>
+      </c>
+      <c r="I73">
+        <v>51.012481733228597</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B74">
         <v>123697</v>
@@ -3091,15 +3535,21 @@
         <v>1</v>
       </c>
       <c r="F74" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G74" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H74">
+        <v>3.9928233944124698</v>
+      </c>
+      <c r="I74">
+        <v>51.152626521244301</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B75">
         <v>121588</v>
@@ -3114,15 +3564,21 @@
         <v>2</v>
       </c>
       <c r="F75" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G75" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H75">
+        <v>3.9638121009624498</v>
+      </c>
+      <c r="I75">
+        <v>51.0218941326901</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B76">
         <v>119973</v>
@@ -3137,15 +3593,21 @@
         <v>2</v>
       </c>
       <c r="F76" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G76" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H76">
+        <v>3.9396138182027598</v>
+      </c>
+      <c r="I76">
+        <v>51.150890357608901</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B77">
         <v>45530</v>
@@ -3160,15 +3622,21 @@
         <v>1</v>
       </c>
       <c r="F77" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G77" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H77">
+        <v>2.8744370421522398</v>
+      </c>
+      <c r="I77">
+        <v>51.186918351856399</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B78">
         <v>164463</v>
@@ -3183,15 +3651,21 @@
         <v>3</v>
       </c>
       <c r="F78" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G78" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H78">
+        <v>4.5754096596986704</v>
+      </c>
+      <c r="I78">
+        <v>51.139638621607702</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B79">
         <v>35327</v>
@@ -3206,15 +3680,21 @@
         <v>2</v>
       </c>
       <c r="F79" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G79" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H79">
+        <v>2.73648087168691</v>
+      </c>
+      <c r="I79">
+        <v>50.957907727918403</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B80">
         <v>35621</v>
@@ -3229,15 +3709,21 @@
         <v>1</v>
       </c>
       <c r="F80" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G80" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H80">
+        <v>2.7394660093875598</v>
+      </c>
+      <c r="I80">
+        <v>50.992466851232201</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B81">
         <v>155019</v>
@@ -3252,15 +3738,21 @@
         <v>4</v>
       </c>
       <c r="F81" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G81" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+      <c r="H81">
+        <v>4.44061009139938</v>
+      </c>
+      <c r="I81">
+        <v>51.229863374033897</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B82">
         <v>131485</v>
@@ -3275,15 +3767,21 @@
         <v>3</v>
       </c>
       <c r="F82" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G82" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="83" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H82">
+        <v>4.1037309567609297</v>
+      </c>
+      <c r="I82">
+        <v>51.2237028130006</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B83">
         <v>41845</v>
@@ -3298,15 +3796,21 @@
         <v>1</v>
       </c>
       <c r="F83" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G83" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H83">
+        <v>2.8234334845351698</v>
+      </c>
+      <c r="I83">
+        <v>51.135160256616302</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B84">
         <v>173653</v>
@@ -3321,15 +3825,21 @@
         <v>1</v>
       </c>
       <c r="F84" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G84" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H84">
+        <v>4.7089920083155903</v>
+      </c>
+      <c r="I84">
+        <v>51.450796469046999</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B85">
         <v>175974</v>
@@ -3344,15 +3854,21 @@
         <v>1</v>
       </c>
       <c r="F85" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G85" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H85">
+        <v>4.7422720590692196</v>
+      </c>
+      <c r="I85">
+        <v>51.437646270246297</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B86">
         <v>95665</v>
@@ -3367,15 +3883,21 @@
         <v>3</v>
       </c>
       <c r="F86" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G86" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="87" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H86">
+        <v>3.59737479780734</v>
+      </c>
+      <c r="I86">
+        <v>50.8371055329781</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B87">
         <v>95665</v>
@@ -3390,15 +3912,21 @@
         <v>3</v>
       </c>
       <c r="F87" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G87" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H87">
+        <v>3.59737479780734</v>
+      </c>
+      <c r="I87">
+        <v>50.8371055329781</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B88">
         <v>246891</v>
@@ -3413,15 +3941,21 @@
         <v>4</v>
       </c>
       <c r="F88" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G88" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H88">
+        <v>5.7491598259143304</v>
+      </c>
+      <c r="I88">
+        <v>51.001242946773097</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B89">
         <v>92747</v>
@@ -3436,15 +3970,21 @@
         <v>4</v>
       </c>
       <c r="F89" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G89" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H89">
+        <v>3.5562542571251101</v>
+      </c>
+      <c r="I89">
+        <v>50.819324329649</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B90">
         <v>109162</v>
@@ -3459,15 +3999,21 @@
         <v>3</v>
       </c>
       <c r="F90" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G90" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H90">
+        <v>3.7866276411597899</v>
+      </c>
+      <c r="I90">
+        <v>51.028298872252797</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B91">
         <v>80278</v>
@@ -3482,15 +4028,21 @@
         <v>4</v>
       </c>
       <c r="F91" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G91" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="92" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H91">
+        <v>3.3801356095019401</v>
+      </c>
+      <c r="I91">
+        <v>50.779196457246897</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B92">
         <v>160003</v>
@@ -3505,15 +4057,21 @@
         <v>2</v>
       </c>
       <c r="F92" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G92" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H92">
+        <v>4.5115610771077801</v>
+      </c>
+      <c r="I92">
+        <v>51.099850457504303</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B93">
         <v>37170</v>
@@ -3528,15 +4086,21 @@
         <v>2</v>
       </c>
       <c r="F93" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G93" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="H93">
+        <v>2.7566000676070299</v>
+      </c>
+      <c r="I93">
+        <v>51.135929773674903</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B94">
         <v>54184</v>
@@ -3551,15 +4115,21 @@
         <v>1</v>
       </c>
       <c r="F94" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G94" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="95" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H94">
+        <v>2.99935642588818</v>
+      </c>
+      <c r="I94">
+        <v>51.148758359432598</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B95">
         <v>171015</v>
@@ -3574,15 +4144,21 @@
         <v>3</v>
       </c>
       <c r="F95" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G95" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H95">
+        <v>4.6692398257223404</v>
+      </c>
+      <c r="I95">
+        <v>51.172541806173697</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B96">
         <v>145377</v>
@@ -3597,15 +4173,21 @@
         <v>4</v>
       </c>
       <c r="F96" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G96" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H96">
+        <v>4.3023894912801897</v>
+      </c>
+      <c r="I96">
+        <v>51.361480387613803</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B97">
         <v>114450</v>
@@ -3620,15 +4202,21 @@
         <v>2</v>
       </c>
       <c r="F97" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G97" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H97">
+        <v>3.8608364564037898</v>
+      </c>
+      <c r="I97">
+        <v>51.136348813860103</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B98">
         <v>77962</v>
@@ -3643,15 +4231,21 @@
         <v>4</v>
       </c>
       <c r="F98" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G98" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H98">
+        <v>3.3447402043646801</v>
+      </c>
+      <c r="I98">
+        <v>50.896675569574299</v>
+      </c>
+    </row>
+    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B99">
         <v>75352</v>
@@ -3666,15 +4260,21 @@
         <v>2</v>
       </c>
       <c r="F99" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G99" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="100" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H99">
+        <v>3.2992818875038599</v>
+      </c>
+      <c r="I99">
+        <v>51.2637094921688</v>
+      </c>
+    </row>
+    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B100">
         <v>146933</v>
@@ -3689,15 +4289,21 @@
         <v>2</v>
       </c>
       <c r="F100" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G100" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="101" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H100">
+        <v>4.3249090672323396</v>
+      </c>
+      <c r="I100">
+        <v>51.166742770137297</v>
+      </c>
+    </row>
+    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B101">
         <v>159722</v>
@@ -3712,15 +4318,21 @@
         <v>3</v>
       </c>
       <c r="F101" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G101" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H101">
+        <v>4.5075315537433402</v>
+      </c>
+      <c r="I101">
+        <v>51.093850761690803</v>
+      </c>
+    </row>
+    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B102">
         <v>38221</v>
@@ -3735,15 +4347,21 @@
         <v>1</v>
       </c>
       <c r="F102" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G102" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H102">
+        <v>2.7720187640070999</v>
+      </c>
+      <c r="I102">
+        <v>51.124244533394901</v>
+      </c>
+    </row>
+    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B103">
         <v>109590</v>
@@ -3758,15 +4376,21 @@
         <v>1</v>
       </c>
       <c r="F103" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G103" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H103">
+        <v>3.7925887026538199</v>
+      </c>
+      <c r="I103">
+        <v>51.039690591712798</v>
+      </c>
+    </row>
+    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B104">
         <v>119847</v>
@@ -3781,15 +4405,21 @@
         <v>1</v>
       </c>
       <c r="F104" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G104" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H104">
+        <v>3.94105739034709</v>
+      </c>
+      <c r="I104">
+        <v>50.796051629952601</v>
+      </c>
+    </row>
+    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B105">
         <v>148146</v>
@@ -3804,15 +4434,21 @@
         <v>5</v>
       </c>
       <c r="F105" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G105" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H105">
+        <v>4.3421742622303201</v>
+      </c>
+      <c r="I105">
+        <v>51.305024307676199</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B106">
         <v>130819</v>
@@ -3827,15 +4463,21 @@
         <v>2</v>
       </c>
       <c r="F106" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G106" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H106">
+        <v>4.0949009069374398</v>
+      </c>
+      <c r="I106">
+        <v>51.103666386303203</v>
+      </c>
+    </row>
+    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B107">
         <v>109687</v>
@@ -3850,15 +4492,21 @@
         <v>3</v>
       </c>
       <c r="F107" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G107" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H107">
+        <v>3.7927911602364301</v>
+      </c>
+      <c r="I107">
+        <v>51.135758095697199</v>
+      </c>
+    </row>
+    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B108">
         <v>189624</v>
@@ -3873,15 +4521,21 @@
         <v>1</v>
       </c>
       <c r="F108" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G108" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H108">
+        <v>4.9356652006117896</v>
+      </c>
+      <c r="I108">
+        <v>51.200568704644397</v>
+      </c>
+    </row>
+    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B109">
         <v>73439</v>
@@ -3896,15 +4550,21 @@
         <v>3</v>
       </c>
       <c r="F109" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G109" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H109">
+        <v>3.27140106810399</v>
+      </c>
+      <c r="I109">
+        <v>51.283733994211701</v>
+      </c>
+    </row>
+    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B110">
         <v>155388</v>
@@ -3919,15 +4579,21 @@
         <v>3</v>
       </c>
       <c r="F110" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G110" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+        <v>64</v>
+      </c>
+      <c r="H110">
+        <v>4.4458887575872801</v>
+      </c>
+      <c r="I110">
+        <v>51.227496078247597</v>
+      </c>
+    </row>
+    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B111">
         <v>125421</v>
@@ -3942,15 +4608,21 @@
         <v>4</v>
       </c>
       <c r="F111" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G111" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H111">
+        <v>4.01855654588101</v>
+      </c>
+      <c r="I111">
+        <v>51.006608036486597</v>
+      </c>
+    </row>
+    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B112">
         <v>205931</v>
@@ -3965,15 +4637,21 @@
         <v>5</v>
       </c>
       <c r="F112" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G112" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="113" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H112">
+        <v>5.16500117057958</v>
+      </c>
+      <c r="I112">
+        <v>50.967660957197403</v>
+      </c>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B113">
         <v>25205</v>
@@ -3988,15 +4666,21 @@
         <v>2</v>
       </c>
       <c r="F113" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G113" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="114" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H113">
+        <v>2.5898806719577201</v>
+      </c>
+      <c r="I113">
+        <v>51.0237137214841</v>
+      </c>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B114">
         <v>124263</v>
@@ -4011,15 +4695,21 @@
         <v>3</v>
       </c>
       <c r="F114" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G114" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H114">
+        <v>4.0008830838076896</v>
+      </c>
+      <c r="I114">
+        <v>51.156427126224003</v>
+      </c>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B115">
         <v>100253</v>
@@ -4034,15 +4724,21 @@
         <v>1</v>
       </c>
       <c r="F115" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G115" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H115">
+        <v>3.6560188781507499</v>
+      </c>
+      <c r="I115">
+        <v>51.265773238240897</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B116">
         <v>114541</v>
@@ -4057,15 +4753,21 @@
         <v>1</v>
       </c>
       <c r="F116" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G116" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+      <c r="H116">
+        <v>3.8613246590725501</v>
+      </c>
+      <c r="I116">
+        <v>51.2112003019366</v>
+      </c>
+    </row>
+    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B117">
         <v>113426</v>
@@ -4080,15 +4782,21 @@
         <v>1</v>
       </c>
       <c r="F117" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G117" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.35">
+        <v>132</v>
+      </c>
+      <c r="H117">
+        <v>3.84535224231634</v>
+      </c>
+      <c r="I117">
+        <v>51.2126318580872</v>
+      </c>
+    </row>
+    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B118">
         <v>26824</v>
@@ -4103,15 +4811,21 @@
         <v>2</v>
       </c>
       <c r="F118" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G118" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H118">
+        <v>2.61197843955784</v>
+      </c>
+      <c r="I118">
+        <v>51.049958975327797</v>
+      </c>
+    </row>
+    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="B119">
         <v>111916</v>
@@ -4126,15 +4840,21 @@
         <v>2</v>
       </c>
       <c r="F119" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G119" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H119">
+        <v>3.8244837570270498</v>
+      </c>
+      <c r="I119">
+        <v>51.149032110074302</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B120">
         <v>130862</v>
@@ -4149,15 +4869,21 @@
         <v>2</v>
       </c>
       <c r="F120" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G120" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H120">
+        <v>4.0958962306449296</v>
+      </c>
+      <c r="I120">
+        <v>51.038157264527896</v>
+      </c>
+    </row>
+    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B121">
         <v>129690</v>
@@ -4172,15 +4898,21 @@
         <v>2</v>
       </c>
       <c r="F121" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G121" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H121">
+        <v>4.0791197683126699</v>
+      </c>
+      <c r="I121">
+        <v>51.048958076971701</v>
+      </c>
+    </row>
+    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B122">
         <v>72117</v>
@@ -4195,15 +4927,21 @@
         <v>2</v>
       </c>
       <c r="F122" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G122" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H122">
+        <v>3.2550648336900498</v>
+      </c>
+      <c r="I122">
+        <v>51.174396693936004</v>
+      </c>
+    </row>
+    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B123">
         <v>42706</v>
@@ -4218,15 +4956,21 @@
         <v>2</v>
       </c>
       <c r="F123" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G123" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H123">
+        <v>2.83476229362202</v>
+      </c>
+      <c r="I123">
+        <v>51.164859932754098</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B124">
         <v>171784</v>
@@ -4241,15 +4985,21 @@
         <v>1</v>
       </c>
       <c r="F124" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G124" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H124">
+        <v>4.6820992300025104</v>
+      </c>
+      <c r="I124">
+        <v>51.449549405162102</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B125">
         <v>173920</v>
@@ -4264,15 +5014,21 @@
         <v>1</v>
       </c>
       <c r="F125" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G125" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H125">
+        <v>4.7127247824167897</v>
+      </c>
+      <c r="I125">
+        <v>51.436279666955002</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B126">
         <v>123017</v>
@@ -4287,15 +5043,21 @@
         <v>1</v>
       </c>
       <c r="F126" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G126" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H126">
+        <v>3.9831839928766302</v>
+      </c>
+      <c r="I126">
+        <v>51.142977520422697</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B127">
         <v>130497</v>
@@ -4310,15 +5072,21 @@
         <v>4</v>
       </c>
       <c r="F127" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G127" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H127">
+        <v>4.0908674778514298</v>
+      </c>
+      <c r="I127">
+        <v>51.008562436223997</v>
+      </c>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B128">
         <v>31680</v>
@@ -4333,15 +5101,21 @@
         <v>2</v>
       </c>
       <c r="F128" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G128" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="129" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H128">
+        <v>2.6811650320205298</v>
+      </c>
+      <c r="I128">
+        <v>51.0522739444284</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B129">
         <v>126822</v>
@@ -4356,15 +5130,21 @@
         <v>3</v>
       </c>
       <c r="F129" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G129" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="130" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H129">
+        <v>4.0371701410426004</v>
+      </c>
+      <c r="I129">
+        <v>51.197414672530101</v>
+      </c>
+    </row>
+    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="B130">
         <v>138525</v>
@@ -4379,15 +5159,21 @@
         <v>4</v>
       </c>
       <c r="F130" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G130" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="131" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H130">
+        <v>4.2044378507419102</v>
+      </c>
+      <c r="I130">
+        <v>51.242248277461897</v>
+      </c>
+    </row>
+    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="B131">
         <v>117376</v>
@@ -4402,15 +5188,21 @@
         <v>1</v>
       </c>
       <c r="F131" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G131" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="132" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H131">
+        <v>3.9025254753347598</v>
+      </c>
+      <c r="I131">
+        <v>51.148062280130802</v>
+      </c>
+    </row>
+    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B132">
         <v>149391</v>
@@ -4425,15 +5217,21 @@
         <v>2</v>
       </c>
       <c r="F132" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G132" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H132">
+        <v>4.3600383780391203</v>
+      </c>
+      <c r="I132">
+        <v>51.236114278614501</v>
+      </c>
+    </row>
+    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B133">
         <v>123196</v>
@@ -4448,15 +5246,21 @@
         <v>2</v>
       </c>
       <c r="F133" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G133" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H133">
+        <v>3.9867104938507198</v>
+      </c>
+      <c r="I133">
+        <v>51.0243346793171</v>
+      </c>
+    </row>
+    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B134">
         <v>120582</v>
@@ -4471,15 +5275,21 @@
         <v>2</v>
       </c>
       <c r="F134" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G134" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H134">
+        <v>3.9483096428682298</v>
+      </c>
+      <c r="I134">
+        <v>51.151784517246298</v>
+      </c>
+    </row>
+    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B135">
         <v>129405</v>
@@ -4494,15 +5304,21 @@
         <v>1</v>
       </c>
       <c r="F135" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G135" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H135">
+        <v>4.0747308913338998</v>
+      </c>
+      <c r="I135">
+        <v>51.100741511249197</v>
+      </c>
+    </row>
+    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B136">
         <v>29539</v>
@@ -4517,15 +5333,21 @@
         <v>1</v>
       </c>
       <c r="F136" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G136" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H136">
+        <v>2.6502053663048102</v>
+      </c>
+      <c r="I136">
+        <v>51.063641087895697</v>
+      </c>
+    </row>
+    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="B137">
         <v>26747</v>
@@ -4540,15 +5362,21 @@
         <v>1</v>
       </c>
       <c r="F137" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G137" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H137">
+        <v>2.61068253962162</v>
+      </c>
+      <c r="I137">
+        <v>51.055217633366503</v>
+      </c>
+    </row>
+    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B138">
         <v>37436</v>
@@ -4563,15 +5391,21 @@
         <v>5</v>
       </c>
       <c r="F138" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G138" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+      <c r="H138">
+        <v>2.7607054406993701</v>
+      </c>
+      <c r="I138">
+        <v>51.1270938666094</v>
+      </c>
+    </row>
+    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="B139">
         <v>30777</v>
@@ -4586,15 +5420,21 @@
         <v>2</v>
       </c>
       <c r="F139" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G139" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H139">
+        <v>2.6676356268555499</v>
+      </c>
+      <c r="I139">
+        <v>51.070097914477302</v>
+      </c>
+    </row>
+    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B140">
         <v>100112</v>
@@ -4609,15 +5449,21 @@
         <v>5</v>
       </c>
       <c r="F140" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G140" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H140">
+        <v>3.6567268667111201</v>
+      </c>
+      <c r="I140">
+        <v>51.0871131329543</v>
+      </c>
+    </row>
+    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B141">
         <v>119218</v>
@@ -4632,15 +5478,21 @@
         <v>1</v>
       </c>
       <c r="F141" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G141" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H141">
+        <v>3.9294586931014601</v>
+      </c>
+      <c r="I141">
+        <v>51.083238606026001</v>
+      </c>
+    </row>
+    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B142">
         <v>142580</v>
@@ -4655,15 +5507,21 @@
         <v>4</v>
       </c>
       <c r="F142" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G142" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H142">
+        <v>4.2623345645251902</v>
+      </c>
+      <c r="I142">
+        <v>51.3173295596335</v>
+      </c>
+    </row>
+    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B143">
         <v>146532</v>
@@ -4678,15 +5536,21 @@
         <v>7</v>
       </c>
       <c r="F143" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G143" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H143">
+        <v>4.3192496508376701</v>
+      </c>
+      <c r="I143">
+        <v>51.0963950677409</v>
+      </c>
+    </row>
+    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B144">
         <v>109713</v>
@@ -4701,15 +5565,21 @@
         <v>2</v>
       </c>
       <c r="F144" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G144" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H144">
+        <v>3.7937036936023198</v>
+      </c>
+      <c r="I144">
+        <v>51.091752312171998</v>
+      </c>
+    </row>
+    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="B145">
         <v>131641</v>
@@ -4724,15 +5594,21 @@
         <v>4</v>
       </c>
       <c r="F145" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G145" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H145">
+        <v>4.10702353180546</v>
+      </c>
+      <c r="I145">
+        <v>51.034443010985299</v>
+      </c>
+    </row>
+    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B146">
         <v>114025</v>
@@ -4747,15 +5623,21 @@
         <v>2</v>
       </c>
       <c r="F146" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G146" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H146">
+        <v>3.8562342418320901</v>
+      </c>
+      <c r="I146">
+        <v>51.002175603778198</v>
+      </c>
+    </row>
+    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B147">
         <v>66112</v>
@@ -4770,15 +5652,21 @@
         <v>2</v>
       </c>
       <c r="F147" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G147" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H147">
+        <v>3.1715586471975801</v>
+      </c>
+      <c r="I147">
+        <v>51.081955505872202</v>
+      </c>
+    </row>
+    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B148">
         <v>155617</v>
@@ -4793,15 +5681,21 @@
         <v>6</v>
       </c>
       <c r="F148" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G148" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H148">
+        <v>4.4488568785209504</v>
+      </c>
+      <c r="I148">
+        <v>51.048565616011302</v>
+      </c>
+    </row>
+    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B149">
         <v>98109</v>
@@ -4816,15 +5710,21 @@
         <v>3</v>
       </c>
       <c r="F149" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G149" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H149">
+        <v>3.6273948150782398</v>
+      </c>
+      <c r="I149">
+        <v>51.134035940570897</v>
+      </c>
+    </row>
+    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="B150">
         <v>97424</v>
@@ -4839,15 +5739,21 @@
         <v>6</v>
       </c>
       <c r="F150" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G150" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="151" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H150">
+        <v>3.6172862407776698</v>
+      </c>
+      <c r="I150">
+        <v>51.154053734170802</v>
+      </c>
+    </row>
+    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B151">
         <v>127820</v>
@@ -4862,15 +5768,21 @@
         <v>3</v>
       </c>
       <c r="F151" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G151" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="152" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H151">
+        <v>4.0520964784137403</v>
+      </c>
+      <c r="I151">
+        <v>51.101626871441098</v>
+      </c>
+    </row>
+    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B152">
         <v>138310</v>
@@ -4885,15 +5797,21 @@
         <v>6</v>
       </c>
       <c r="F152" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G152" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="153" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H152">
+        <v>4.2013165499801399</v>
+      </c>
+      <c r="I152">
+        <v>51.254135455586102</v>
+      </c>
+    </row>
+    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B153">
         <v>122696</v>
@@ -4908,15 +5826,21 @@
         <v>3</v>
       </c>
       <c r="F153" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G153" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="154" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H153">
+        <v>3.9787120226916199</v>
+      </c>
+      <c r="I153">
+        <v>51.129183025299803</v>
+      </c>
+    </row>
+    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B154">
         <v>51287</v>
@@ -4931,15 +5855,21 @@
         <v>2</v>
       </c>
       <c r="F154" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G154" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="155" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H154">
+        <v>2.96169292631865</v>
+      </c>
+      <c r="I154">
+        <v>51.024400293541703</v>
+      </c>
+    </row>
+    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B155">
         <v>118746</v>
@@ -4954,15 +5884,21 @@
         <v>4</v>
       </c>
       <c r="F155" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G155" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="156" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H155">
+        <v>3.9233388498073798</v>
+      </c>
+      <c r="I155">
+        <v>51.018431184812698</v>
+      </c>
+    </row>
+    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B156">
         <v>43886</v>
@@ -4977,15 +5913,21 @@
         <v>1</v>
       </c>
       <c r="F156" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G156" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="157" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H156">
+        <v>2.8515140138383401</v>
+      </c>
+      <c r="I156">
+        <v>51.168591537295299</v>
+      </c>
+    </row>
+    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B157">
         <v>244241</v>
@@ -5000,15 +5942,21 @@
         <v>0</v>
       </c>
       <c r="F157" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G157" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="158" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H157">
+        <v>5.7162152322012902</v>
+      </c>
+      <c r="I157">
+        <v>51.168521269219099</v>
+      </c>
+    </row>
+    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B158">
         <v>41947</v>
@@ -5023,15 +5971,21 @@
         <v>2</v>
       </c>
       <c r="F158" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G158" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="159" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H158">
+        <v>2.8293105495496</v>
+      </c>
+      <c r="I158">
+        <v>51.001004063471299</v>
+      </c>
+    </row>
+    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B159">
         <v>243534</v>
@@ -5046,15 +6000,21 @@
         <v>0</v>
       </c>
       <c r="F159" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G159" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="160" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H159">
+        <v>5.7058189702372699</v>
+      </c>
+      <c r="I159">
+        <v>51.158525700450298</v>
+      </c>
+    </row>
+    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B160">
         <v>159015</v>
@@ -5069,15 +6029,21 @@
         <v>1</v>
       </c>
       <c r="F160" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G160" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="161" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H160">
+        <v>4.4974219704417102</v>
+      </c>
+      <c r="I160">
+        <v>51.087498190970997</v>
+      </c>
+    </row>
+    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B161">
         <v>146160</v>
@@ -5092,15 +6058,21 @@
         <v>3</v>
       </c>
       <c r="F161" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G161" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="162" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H161">
+        <v>4.3139177238320601</v>
+      </c>
+      <c r="I161">
+        <v>51.115017484514198</v>
+      </c>
+    </row>
+    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B162">
         <v>35440</v>
@@ -5115,15 +6087,21 @@
         <v>1</v>
       </c>
       <c r="F162" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G162" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="163" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H162">
+        <v>2.7329169321584699</v>
+      </c>
+      <c r="I162">
+        <v>51.106230683744897</v>
+      </c>
+    </row>
+    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B163">
         <v>35426</v>
@@ -5138,15 +6116,21 @@
         <v>1</v>
       </c>
       <c r="F163" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G163" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="164" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H163">
+        <v>2.73273312264415</v>
+      </c>
+      <c r="I163">
+        <v>51.1057695962173</v>
+      </c>
+    </row>
+    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="B164">
         <v>34428</v>
@@ -5161,15 +6145,21 @@
         <v>1</v>
       </c>
       <c r="F164" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G164" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="165" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H164">
+        <v>2.7189684944569499</v>
+      </c>
+      <c r="I164">
+        <v>51.091929549221398</v>
+      </c>
+    </row>
+    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B165">
         <v>33164</v>
@@ -5184,15 +6174,21 @@
         <v>1</v>
       </c>
       <c r="F165" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G165" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="166" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H165">
+        <v>2.7026947834869302</v>
+      </c>
+      <c r="I165">
+        <v>51.042159494521897</v>
+      </c>
+    </row>
+    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B166">
         <v>120307</v>
@@ -5207,15 +6203,21 @@
         <v>2</v>
       </c>
       <c r="F166" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G166" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="167" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H166">
+        <v>3.9475372055906002</v>
+      </c>
+      <c r="I166">
+        <v>50.801082372254399</v>
+      </c>
+    </row>
+    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B167">
         <v>47303</v>
@@ -5230,15 +6232,21 @@
         <v>1</v>
       </c>
       <c r="F167" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G167" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="168" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H167">
+        <v>2.9019962117914502</v>
+      </c>
+      <c r="I167">
+        <v>51.1170577331456</v>
+      </c>
+    </row>
+    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B168">
         <v>127578</v>
@@ -5253,15 +6261,21 @@
         <v>2</v>
       </c>
       <c r="F168" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G168" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="169" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H168">
+        <v>4.0490270076585304</v>
+      </c>
+      <c r="I168">
+        <v>51.045131989693097</v>
+      </c>
+    </row>
+    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B169">
         <v>126695</v>
@@ -5276,15 +6290,21 @@
         <v>3</v>
       </c>
       <c r="F169" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G169" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="170" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H169">
+        <v>4.0360878777881304</v>
+      </c>
+      <c r="I169">
+        <v>51.094176050107301</v>
+      </c>
+    </row>
+    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B170">
         <v>48246</v>
@@ -5299,15 +6319,21 @@
         <v>1</v>
       </c>
       <c r="F170" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G170" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="171" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H170">
+        <v>2.91481766287112</v>
+      </c>
+      <c r="I170">
+        <v>51.137912352329799</v>
+      </c>
+    </row>
+    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B171">
         <v>148747</v>
@@ -5322,15 +6348,21 @@
         <v>6</v>
       </c>
       <c r="F171" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G171" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="172" spans="1:7" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+      <c r="H171">
+        <v>4.3508735627312198</v>
+      </c>
+      <c r="I171">
+        <v>51.084367883504299</v>
+      </c>
+    </row>
+    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B172">
         <v>44973</v>
@@ -5345,15 +6377,21 @@
         <v>2</v>
       </c>
       <c r="F172" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G172" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="173" spans="1:7" x14ac:dyDescent="0.35">
+        <v>13</v>
+      </c>
+      <c r="H172">
+        <v>2.86892119210356</v>
+      </c>
+      <c r="I172">
+        <v>51.110591348442298</v>
+      </c>
+    </row>
+    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B173">
         <v>77796</v>
@@ -5368,10 +6406,16 @@
         <v>2</v>
       </c>
       <c r="F173" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G173" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="H173">
+        <v>3.34396975363327</v>
+      </c>
+      <c r="I173">
+        <v>50.823802199200998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>